<commit_message>
Actualiza tablas de data: equiv_conceptos formato nuevo, cot_afp_hist y parametros mensuales
</commit_message>
<xml_diff>
--- a/data/cot_afp_hist.xlsx
+++ b/data/cot_afp_hist.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_Ia\Version20\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_Ia\rex-tools-hub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25489DBD-DFDC-48E7-AF5C-3AC00446B836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D376164B-B795-4E6D-8CA6-83244C2E896E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2925" yWindow="0" windowWidth="15375" windowHeight="12705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$F$204</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1210,6 +1210,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F226"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1242,7 +1243,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -1262,7 +1263,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>44</v>
       </c>
@@ -1282,7 +1283,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>45</v>
       </c>
@@ -1302,7 +1303,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>46</v>
       </c>
@@ -1322,7 +1323,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -1342,7 +1343,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>48</v>
       </c>
@@ -1362,7 +1363,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>49</v>
       </c>
@@ -1382,7 +1383,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -1402,7 +1403,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>51</v>
       </c>
@@ -1422,7 +1423,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>52</v>
       </c>
@@ -1442,7 +1443,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>53</v>
       </c>
@@ -1462,7 +1463,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>54</v>
       </c>
@@ -1482,7 +1483,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>55</v>
       </c>
@@ -1502,7 +1503,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>56</v>
       </c>
@@ -1522,7 +1523,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>57</v>
       </c>
@@ -1542,7 +1543,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>58</v>
       </c>
@@ -1562,7 +1563,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>59</v>
       </c>
@@ -1582,7 +1583,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>60</v>
       </c>
@@ -1602,7 +1603,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>61</v>
       </c>
@@ -1622,7 +1623,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>62</v>
       </c>
@@ -1642,7 +1643,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>63</v>
       </c>
@@ -1662,7 +1663,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>64</v>
       </c>
@@ -1682,7 +1683,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -1702,7 +1703,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>66</v>
       </c>
@@ -1722,7 +1723,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -1742,7 +1743,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>68</v>
       </c>
@@ -1762,7 +1763,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>69</v>
       </c>
@@ -1782,7 +1783,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>70</v>
       </c>
@@ -1802,7 +1803,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>71</v>
       </c>
@@ -1822,7 +1823,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>72</v>
       </c>
@@ -1842,7 +1843,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>73</v>
       </c>
@@ -1862,7 +1863,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>74</v>
       </c>
@@ -1882,7 +1883,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>75</v>
       </c>
@@ -1902,7 +1903,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>76</v>
       </c>
@@ -1922,7 +1923,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>77</v>
       </c>
@@ -1942,7 +1943,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>78</v>
       </c>
@@ -1962,7 +1963,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>79</v>
       </c>
@@ -1982,7 +1983,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>80</v>
       </c>
@@ -2002,7 +2003,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>81</v>
       </c>
@@ -2022,7 +2023,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>82</v>
       </c>
@@ -2042,7 +2043,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>83</v>
       </c>
@@ -2062,7 +2063,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>84</v>
       </c>
@@ -2082,7 +2083,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>85</v>
       </c>
@@ -2102,7 +2103,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>86</v>
       </c>
@@ -2122,7 +2123,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>87</v>
       </c>
@@ -2142,7 +2143,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>88</v>
       </c>
@@ -2162,7 +2163,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>89</v>
       </c>
@@ -2182,7 +2183,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>90</v>
       </c>
@@ -2202,7 +2203,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>91</v>
       </c>
@@ -2222,7 +2223,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>92</v>
       </c>
@@ -2242,7 +2243,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>93</v>
       </c>
@@ -2262,7 +2263,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>94</v>
       </c>
@@ -2282,7 +2283,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>95</v>
       </c>
@@ -2302,7 +2303,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>96</v>
       </c>
@@ -2322,7 +2323,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>97</v>
       </c>
@@ -2342,7 +2343,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>98</v>
       </c>
@@ -2362,7 +2363,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>99</v>
       </c>
@@ -2382,7 +2383,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>100</v>
       </c>
@@ -2402,7 +2403,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>101</v>
       </c>
@@ -2422,7 +2423,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>102</v>
       </c>
@@ -2442,7 +2443,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>103</v>
       </c>
@@ -2462,7 +2463,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>104</v>
       </c>
@@ -2482,7 +2483,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>105</v>
       </c>
@@ -2502,7 +2503,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>106</v>
       </c>
@@ -2522,7 +2523,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>107</v>
       </c>
@@ -2542,7 +2543,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>108</v>
       </c>
@@ -2562,7 +2563,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>109</v>
       </c>
@@ -2582,7 +2583,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>110</v>
       </c>
@@ -2602,7 +2603,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>111</v>
       </c>
@@ -2622,7 +2623,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>112</v>
       </c>
@@ -2642,7 +2643,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>113</v>
       </c>
@@ -2662,7 +2663,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>114</v>
       </c>
@@ -2682,7 +2683,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>115</v>
       </c>
@@ -2702,7 +2703,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>116</v>
       </c>
@@ -2722,7 +2723,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>117</v>
       </c>
@@ -2742,7 +2743,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>118</v>
       </c>
@@ -2762,7 +2763,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>119</v>
       </c>
@@ -2782,7 +2783,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>120</v>
       </c>
@@ -2802,7 +2803,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>121</v>
       </c>
@@ -2822,7 +2823,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>122</v>
       </c>
@@ -2842,7 +2843,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>123</v>
       </c>
@@ -2862,7 +2863,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>124</v>
       </c>
@@ -2882,7 +2883,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>125</v>
       </c>
@@ -2902,7 +2903,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>126</v>
       </c>
@@ -2922,7 +2923,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>127</v>
       </c>
@@ -2942,7 +2943,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>128</v>
       </c>
@@ -2962,7 +2963,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>129</v>
       </c>
@@ -2982,7 +2983,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>130</v>
       </c>
@@ -3002,7 +3003,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>131</v>
       </c>
@@ -3022,7 +3023,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>132</v>
       </c>
@@ -3042,7 +3043,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>133</v>
       </c>
@@ -3062,7 +3063,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>134</v>
       </c>
@@ -3082,7 +3083,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>135</v>
       </c>
@@ -3102,7 +3103,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>136</v>
       </c>
@@ -3122,7 +3123,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>137</v>
       </c>
@@ -3142,7 +3143,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>138</v>
       </c>
@@ -3162,7 +3163,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>139</v>
       </c>
@@ -3182,7 +3183,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>140</v>
       </c>
@@ -3202,7 +3203,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>141</v>
       </c>
@@ -3222,7 +3223,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>142</v>
       </c>
@@ -3242,7 +3243,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>143</v>
       </c>
@@ -3262,7 +3263,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>144</v>
       </c>
@@ -3282,7 +3283,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>145</v>
       </c>
@@ -3302,7 +3303,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>146</v>
       </c>
@@ -3322,7 +3323,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>147</v>
       </c>
@@ -3342,7 +3343,7 @@
         <v>1.38E-2</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>148</v>
       </c>
@@ -3362,7 +3363,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>149</v>
       </c>
@@ -3382,7 +3383,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>150</v>
       </c>
@@ -3402,7 +3403,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>151</v>
       </c>
@@ -3422,7 +3423,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>152</v>
       </c>
@@ -3442,7 +3443,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>153</v>
       </c>
@@ -3462,7 +3463,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>154</v>
       </c>
@@ -3482,7 +3483,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>155</v>
       </c>
@@ -3502,7 +3503,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>156</v>
       </c>
@@ -3522,7 +3523,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>157</v>
       </c>
@@ -3542,7 +3543,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>158</v>
       </c>
@@ -3562,7 +3563,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>159</v>
       </c>
@@ -3582,7 +3583,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>160</v>
       </c>
@@ -3602,7 +3603,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>161</v>
       </c>
@@ -3622,7 +3623,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>162</v>
       </c>
@@ -3642,7 +3643,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>163</v>
       </c>
@@ -3662,7 +3663,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>164</v>
       </c>
@@ -3682,7 +3683,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>165</v>
       </c>
@@ -3702,7 +3703,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>166</v>
       </c>
@@ -3722,7 +3723,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>167</v>
       </c>
@@ -3742,7 +3743,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>168</v>
       </c>
@@ -3762,7 +3763,7 @@
         <v>1.78E-2</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>169</v>
       </c>
@@ -3782,7 +3783,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>170</v>
       </c>
@@ -3802,7 +3803,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>171</v>
       </c>
@@ -3822,7 +3823,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>172</v>
       </c>
@@ -3842,7 +3843,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>173</v>
       </c>
@@ -3862,7 +3863,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>174</v>
       </c>
@@ -3882,7 +3883,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>175</v>
       </c>
@@ -3902,7 +3903,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>182</v>
       </c>
@@ -3922,7 +3923,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>183</v>
       </c>
@@ -3942,7 +3943,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>184</v>
       </c>
@@ -3962,7 +3963,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>185</v>
       </c>
@@ -3982,7 +3983,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>186</v>
       </c>
@@ -4002,7 +4003,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>187</v>
       </c>
@@ -4022,7 +4023,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>188</v>
       </c>
@@ -4042,7 +4043,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>189</v>
       </c>
@@ -4062,7 +4063,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>190</v>
       </c>
@@ -4082,7 +4083,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>191</v>
       </c>
@@ -4102,7 +4103,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>192</v>
       </c>
@@ -4122,7 +4123,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>193</v>
       </c>
@@ -4142,7 +4143,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>194</v>
       </c>
@@ -4162,7 +4163,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>195</v>
       </c>
@@ -4182,7 +4183,7 @@
         <v>1.8800000000000001E-2</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>196</v>
       </c>
@@ -4202,7 +4203,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>197</v>
       </c>
@@ -4222,7 +4223,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>198</v>
       </c>
@@ -4242,7 +4243,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>199</v>
       </c>
@@ -4262,7 +4263,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>200</v>
       </c>
@@ -4282,7 +4283,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>201</v>
       </c>
@@ -4302,7 +4303,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>202</v>
       </c>
@@ -4322,7 +4323,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>203</v>
       </c>
@@ -4342,7 +4343,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>204</v>
       </c>
@@ -4362,7 +4363,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>205</v>
       </c>
@@ -4382,7 +4383,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>206</v>
       </c>
@@ -4402,7 +4403,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>207</v>
       </c>
@@ -4422,7 +4423,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>208</v>
       </c>
@@ -4442,7 +4443,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>209</v>
       </c>
@@ -4462,7 +4463,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>210</v>
       </c>
@@ -4482,7 +4483,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>211</v>
       </c>
@@ -4502,7 +4503,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>212</v>
       </c>
@@ -4522,7 +4523,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>213</v>
       </c>
@@ -4542,7 +4543,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>214</v>
       </c>
@@ -4562,7 +4563,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>215</v>
       </c>
@@ -4582,7 +4583,7 @@
         <v>1.49E-2</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>216</v>
       </c>
@@ -5723,7 +5724,47 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F204" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="2026-01capital"/>
+        <filter val="2026-01cuprum"/>
+        <filter val="2026-01habitat"/>
+        <filter val="2026-01modelo"/>
+        <filter val="2026-01planvital"/>
+        <filter val="2026-01provida"/>
+        <filter val="2026-01uno"/>
+        <filter val="2026-02capital"/>
+        <filter val="2026-02cuprum"/>
+        <filter val="2026-02habitat"/>
+        <filter val="2026-02modelo"/>
+        <filter val="2026-02planvital"/>
+        <filter val="2026-02provida"/>
+        <filter val="2026-02uno"/>
+        <filter val="2026-03capital"/>
+        <filter val="2026-03cuprum"/>
+        <filter val="2026-03habitat"/>
+        <filter val="2026-03modelo"/>
+        <filter val="2026-03planvital"/>
+        <filter val="2026-03provida"/>
+        <filter val="2026-03uno"/>
+        <filter val="2026-04capital"/>
+        <filter val="2026-04cuprum"/>
+        <filter val="2026-04habitat"/>
+        <filter val="2026-04modelo"/>
+        <filter val="2026-04planvital"/>
+        <filter val="2026-04provida"/>
+        <filter val="2026-04uno"/>
+        <filter val="2026-05capital"/>
+        <filter val="2026-05cuprum"/>
+        <filter val="2026-05habitat"/>
+        <filter val="2026-05modelo"/>
+        <filter val="2026-05planvital"/>
+        <filter val="2026-05provida"/>
+        <filter val="2026-05uno"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>